<commit_message>
Add Sales + Service Purchase Register consolidation before ITC matching.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/samples/sample_purchase_register.xlsx
+++ b/samples/sample_purchase_register.xlsx
@@ -500,74 +500,74 @@
         <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E4">
-        <v>25000</v>
+        <v>100000</v>
       </c>
       <c r="F4">
         <v>0</v>
       </c>
       <c r="G4">
-        <v>2250</v>
+        <v>9000</v>
       </c>
       <c r="H4">
-        <v>2250</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E5">
-        <v>30000</v>
+        <v>25000</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
       <c r="G5">
-        <v>2700</v>
+        <v>2250</v>
       </c>
       <c r="H5">
-        <v>2700</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E6">
-        <v>100000</v>
+        <v>30000</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="G6">
-        <v>9000</v>
+        <v>2700</v>
       </c>
       <c r="H6">
-        <v>9000</v>
+        <v>2700</v>
       </c>
     </row>
   </sheetData>

</xml_diff>